<commit_message>
Afegir rol nou-incorporat: nous professionals cobreixen Dc 16-20 en rotació
- planning_generator.py: nova cua separada per nou-incorporats a Config; algorisme prioritza aquesta cua per als torns de dimecres 16-20 (excepte 1r Dc del mes)
- validate_planning: nova validació que assegura nou-incorporats només al seu torn
- app.py: mostra els nou-incorporats a l'expander de configuració detectada
- 02_Plantilla_Entrada.xlsx: opció 'nou-incorporat' afegida a la validació del camp Rol + notes a Instruccions i Radiòlegs
- 01_Regles_Procés.docx: v2.1 amb el nou rol documentat
- EXEMPLE + Benchmark: mostra 2 nou-incorporats de demo (Novell-Nou1, Novell-Nou2)
- README: nova secció explicativa
</commit_message>
<xml_diff>
--- a/02_Plantilla_Entrada.xlsx
+++ b/02_Plantilla_Entrada.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,6 +66,11 @@
     <font>
       <i val="1"/>
       <color rgb="00888888"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -122,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,6 +149,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -509,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -694,6 +700,34 @@
       <c r="A30" s="1" t="inlineStr">
         <is>
           <t>IMPORTANT: Aquesta plantilla NO conté noms preinstal·lats. Has de poblar-la amb la teva plantilla real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>ACTUALITZACIÓ: nou rol "nou-incorporat"</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Quan un radiòleg s'incorpora nou a Telediagnòstic, marca'l amb el rol "nou-incorporat" a la pestanya Radiòlegs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Aquests professionals cobriran els torns de dimecres 16-20 (excepte el 1r dimecres del mes, que és fix).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Si hi ha diversos nou-incorporats, rotaran entre ells per als dimecres tarda. Quan es considerin formats, canvieu el rol a "rotador".</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1429,6 +1463,8 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="6" t="n"/>
     </row>
+    <row r="54"/>
+    <row r="55"/>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
@@ -1442,6 +1478,7 @@
           <t>rotador</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr"/>
       <c r="C57" s="12" t="inlineStr">
         <is>
           <t>Participa a la roda alfabètica de guàrdies. Cas habitual per a la majoria.</t>
@@ -1454,6 +1491,7 @@
           <t>fix-només</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr"/>
       <c r="C58" s="12" t="inlineStr">
         <is>
           <t>Només cobreix els seus torns fixos definits a Configuració. No participa a la roda.</t>
@@ -1466,6 +1504,7 @@
           <t>fix-i-rota</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr"/>
       <c r="C59" s="12" t="inlineStr">
         <is>
           <t>Té torns fixos però també participa a la roda per a guàrdies addicionals.</t>
@@ -1478,6 +1517,7 @@
           <t>sun-nit-only</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr"/>
       <c r="C60" s="12" t="inlineStr">
         <is>
           <t>Cas especial: només fa guàrdies de diumenge nit. Vegeu Configuració.</t>
@@ -1490,9 +1530,23 @@
           <t>weekend-day-only</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr"/>
       <c r="C61" s="12" t="inlineStr">
         <is>
           <t>Cas especial: només dissabte/diumenge dia. Vegeu Configuració.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>nou-incorporat</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>Nou professional en període de rodatge: només cobreix dimecres 16-20 (excepte 1r Dc del mes). Quan es consideri format, canvieu-li el rol a "rotador".</t>
         </is>
       </c>
     </row>
@@ -1501,8 +1555,8 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B4:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Valor no vàlid" promptTitle="Rol del professional" prompt="rotador = participa a la roda alfabètica&#10;fix-només = només cobreix torns fixos, no rota&#10;fix-i-rota = té torn fix però també participa a la roda&#10;sun-nit-only = només diumenge nit&#10;weekend-day-only = només dissabte/diumenge dia" type="list">
-      <formula1>"rotador,fix-només,fix-i-rota,sun-nit-only,weekend-day-only"</formula1>
+    <dataValidation sqref="B4:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Valor no vàlid" promptTitle="Rol del professional" prompt="rotador = participa a la roda alfabètica&#10;fix-només = només cobreix torns fixos, no rota&#10;fix-i-rota = té torn fix però també participa a la roda&#10;sun-nit-only = només diumenge nit&#10;weekend-day-only = només dissabte/diumenge dia&#10;nou-incorporat = només dimecres 16-20 (excepte 1r del mes)" type="list">
+      <formula1>"rotador,fix-només,fix-i-rota,sun-nit-only,weekend-day-only,nou-incorporat"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>